<commit_message>
deploy: update local database binary and tax dataset parameters
</commit_message>
<xml_diff>
--- a/datasets/tax_dataset.xlsx
+++ b/datasets/tax_dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Major_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MAJOR PROJECT\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6550ED-D6C4-4390-9722-86D748D89F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C81198-E211-431D-BA6B-C32268A2C2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{693A3F0A-E8AB-4656-A4EB-F60B1E96A312}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{693A3F0A-E8AB-4656-A4EB-F60B1E96A312}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -2749,7 +2740,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2846,7 +2837,7 @@
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2867,9 +2858,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2907,7 +2898,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3013,7 +3004,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3155,7 +3146,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3164,7 +3155,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C640C34-28F8-4BB4-B668-EE4764BD9A88}">
   <dimension ref="A1:G483"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
     <col min="2" max="2" width="40.77734375" customWidth="1"/>
@@ -3174,7 +3165,7 @@
     <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="5" customFormat="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3194,7 +3185,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3214,7 +3205,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -3234,7 +3225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3254,7 +3245,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3274,7 +3265,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -3294,7 +3285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -3314,7 +3305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -3334,7 +3325,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -3354,7 +3345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -3374,7 +3365,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -3394,7 +3385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -3414,7 +3405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -3434,7 +3425,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -3454,7 +3445,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -3474,7 +3465,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -3494,7 +3485,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -3514,7 +3505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -3534,7 +3525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -3554,7 +3545,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -3574,7 +3565,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -3594,7 +3585,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -3614,7 +3605,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -3634,7 +3625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -3654,7 +3645,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -3674,7 +3665,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -3694,7 +3685,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -3714,7 +3705,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -3734,7 +3725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -3754,7 +3745,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -3774,7 +3765,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -3794,7 +3785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -3814,7 +3805,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -3834,7 +3825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -3854,7 +3845,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -3874,7 +3865,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -3894,7 +3885,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -3914,7 +3905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -3934,7 +3925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -3954,7 +3945,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -3974,7 +3965,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -3994,7 +3985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -4014,7 +4005,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -4034,7 +4025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -4054,7 +4045,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -4074,7 +4065,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -4094,7 +4085,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -4114,7 +4105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -4134,7 +4125,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -4154,7 +4145,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -4174,7 +4165,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -4194,7 +4185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -4214,7 +4205,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>57</v>
       </c>
@@ -4234,7 +4225,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -4254,7 +4245,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -4274,7 +4265,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -4294,7 +4285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>61</v>
       </c>
@@ -4314,7 +4305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>62</v>
       </c>
@@ -4334,7 +4325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>63</v>
       </c>
@@ -4354,7 +4345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -4374,7 +4365,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>65</v>
       </c>
@@ -4394,7 +4385,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -4414,7 +4405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -4434,7 +4425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -4454,7 +4445,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -4474,7 +4465,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7">
       <c r="A66" t="s">
         <v>70</v>
       </c>
@@ -4494,7 +4485,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -4514,7 +4505,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7">
       <c r="A68" t="s">
         <v>72</v>
       </c>
@@ -4534,7 +4525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7">
       <c r="A69" t="s">
         <v>73</v>
       </c>
@@ -4554,7 +4545,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7">
       <c r="A70" t="s">
         <v>74</v>
       </c>
@@ -4574,7 +4565,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7">
       <c r="A71" t="s">
         <v>75</v>
       </c>
@@ -4594,7 +4585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7">
       <c r="A72" t="s">
         <v>76</v>
       </c>
@@ -4614,7 +4605,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7">
       <c r="A73" t="s">
         <v>77</v>
       </c>
@@ -4634,7 +4625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7">
       <c r="A74" t="s">
         <v>78</v>
       </c>
@@ -4654,7 +4645,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -4674,7 +4665,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7">
       <c r="A76" t="s">
         <v>80</v>
       </c>
@@ -4694,7 +4685,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7">
       <c r="A77" t="s">
         <v>81</v>
       </c>
@@ -4714,7 +4705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7">
       <c r="A78" t="s">
         <v>82</v>
       </c>
@@ -4734,7 +4725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -4754,7 +4745,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7">
       <c r="A80" t="s">
         <v>84</v>
       </c>
@@ -4774,7 +4765,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7">
       <c r="A81" t="s">
         <v>85</v>
       </c>
@@ -4794,7 +4785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7">
       <c r="A82" t="s">
         <v>86</v>
       </c>
@@ -4814,7 +4805,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7">
       <c r="A83" t="s">
         <v>87</v>
       </c>
@@ -4834,7 +4825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7">
       <c r="A84" t="s">
         <v>88</v>
       </c>
@@ -4854,7 +4845,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7">
       <c r="A85" t="s">
         <v>89</v>
       </c>
@@ -4874,7 +4865,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7">
       <c r="A86" t="s">
         <v>90</v>
       </c>
@@ -4894,7 +4885,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7">
       <c r="A87" t="s">
         <v>91</v>
       </c>
@@ -4914,7 +4905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7">
       <c r="A88" t="s">
         <v>92</v>
       </c>
@@ -4934,7 +4925,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7">
       <c r="A89" t="s">
         <v>93</v>
       </c>
@@ -4954,7 +4945,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7">
       <c r="A90" t="s">
         <v>94</v>
       </c>
@@ -4974,7 +4965,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7">
       <c r="A91" t="s">
         <v>95</v>
       </c>
@@ -4994,7 +4985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7">
       <c r="A92" t="s">
         <v>96</v>
       </c>
@@ -5014,7 +5005,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7">
       <c r="A93" t="s">
         <v>97</v>
       </c>
@@ -5034,7 +5025,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7">
       <c r="A94" t="s">
         <v>98</v>
       </c>
@@ -5054,7 +5045,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7">
       <c r="A95" t="s">
         <v>99</v>
       </c>
@@ -5074,7 +5065,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7">
       <c r="A96" t="s">
         <v>100</v>
       </c>
@@ -5094,7 +5085,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7">
       <c r="A97" t="s">
         <v>101</v>
       </c>
@@ -5114,7 +5105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7">
       <c r="A98" t="s">
         <v>102</v>
       </c>
@@ -5134,7 +5125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7">
       <c r="A99" t="s">
         <v>103</v>
       </c>
@@ -5154,7 +5145,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7">
       <c r="A100" t="s">
         <v>104</v>
       </c>
@@ -5174,7 +5165,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7">
       <c r="A101" t="s">
         <v>105</v>
       </c>
@@ -5194,7 +5185,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7">
       <c r="A102" t="s">
         <v>106</v>
       </c>
@@ -5214,7 +5205,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7">
       <c r="A103" t="s">
         <v>107</v>
       </c>
@@ -5234,7 +5225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7">
       <c r="A104" t="s">
         <v>108</v>
       </c>
@@ -5254,7 +5245,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7">
       <c r="A105" t="s">
         <v>109</v>
       </c>
@@ -5274,7 +5265,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7">
       <c r="A106" t="s">
         <v>110</v>
       </c>
@@ -5294,7 +5285,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7">
       <c r="A107" t="s">
         <v>111</v>
       </c>
@@ -5314,7 +5305,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7">
       <c r="A108" t="s">
         <v>112</v>
       </c>
@@ -5334,7 +5325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7">
       <c r="A109" t="s">
         <v>113</v>
       </c>
@@ -5354,7 +5345,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7">
       <c r="A110" t="s">
         <v>114</v>
       </c>
@@ -5374,7 +5365,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7">
       <c r="A111" t="s">
         <v>115</v>
       </c>
@@ -5394,7 +5385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7">
       <c r="A112" t="s">
         <v>116</v>
       </c>
@@ -5414,7 +5405,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7">
       <c r="A113" t="s">
         <v>117</v>
       </c>
@@ -5434,7 +5425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7">
       <c r="A114" t="s">
         <v>118</v>
       </c>
@@ -5454,7 +5445,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7">
       <c r="A115" t="s">
         <v>119</v>
       </c>
@@ -5474,7 +5465,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7">
       <c r="A116" t="s">
         <v>120</v>
       </c>
@@ -5494,7 +5485,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7">
       <c r="A117" t="s">
         <v>121</v>
       </c>
@@ -5514,7 +5505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7">
       <c r="A118" t="s">
         <v>122</v>
       </c>
@@ -5534,7 +5525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7">
       <c r="A119" t="s">
         <v>123</v>
       </c>
@@ -5554,7 +5545,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7">
       <c r="A120" t="s">
         <v>124</v>
       </c>
@@ -5574,7 +5565,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7">
       <c r="A121" t="s">
         <v>125</v>
       </c>
@@ -5594,7 +5585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7">
       <c r="A122" t="s">
         <v>126</v>
       </c>
@@ -5614,7 +5605,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7">
       <c r="A123" t="s">
         <v>127</v>
       </c>
@@ -5634,7 +5625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7">
       <c r="A124" t="s">
         <v>128</v>
       </c>
@@ -5654,7 +5645,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7">
       <c r="A125" t="s">
         <v>129</v>
       </c>
@@ -5674,7 +5665,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7">
       <c r="A126" t="s">
         <v>130</v>
       </c>
@@ -5694,7 +5685,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7">
       <c r="A127" t="s">
         <v>131</v>
       </c>
@@ -5714,7 +5705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7">
       <c r="A128" t="s">
         <v>132</v>
       </c>
@@ -5734,7 +5725,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7">
       <c r="A129" t="s">
         <v>133</v>
       </c>
@@ -5754,7 +5745,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7">
       <c r="A130" t="s">
         <v>134</v>
       </c>
@@ -5774,7 +5765,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7">
       <c r="A131" t="s">
         <v>135</v>
       </c>
@@ -5794,7 +5785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7">
       <c r="A132" t="s">
         <v>136</v>
       </c>
@@ -5814,7 +5805,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7">
       <c r="A133" t="s">
         <v>137</v>
       </c>
@@ -5834,7 +5825,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7">
       <c r="A134" t="s">
         <v>138</v>
       </c>
@@ -5854,7 +5845,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7">
       <c r="A135" t="s">
         <v>139</v>
       </c>
@@ -5874,7 +5865,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7">
       <c r="A136" t="s">
         <v>140</v>
       </c>
@@ -5894,7 +5885,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:7">
       <c r="A137" t="s">
         <v>141</v>
       </c>
@@ -5914,7 +5905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:7">
       <c r="A138" t="s">
         <v>142</v>
       </c>
@@ -5934,7 +5925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7">
       <c r="A139" t="s">
         <v>143</v>
       </c>
@@ -5954,7 +5945,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:7">
       <c r="A140" t="s">
         <v>144</v>
       </c>
@@ -5974,7 +5965,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:7">
       <c r="A141" t="s">
         <v>145</v>
       </c>
@@ -5994,7 +5985,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7">
       <c r="A142" t="s">
         <v>146</v>
       </c>
@@ -6014,7 +6005,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:7">
       <c r="A143" t="s">
         <v>147</v>
       </c>
@@ -6034,7 +6025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:7">
       <c r="A144" t="s">
         <v>148</v>
       </c>
@@ -6054,7 +6045,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:7">
       <c r="A145" t="s">
         <v>149</v>
       </c>
@@ -6074,7 +6065,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:7">
       <c r="A146" t="s">
         <v>150</v>
       </c>
@@ -6094,7 +6085,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:7">
       <c r="A147" t="s">
         <v>151</v>
       </c>
@@ -6114,7 +6105,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7">
       <c r="A148" t="s">
         <v>152</v>
       </c>
@@ -6134,7 +6125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:7">
       <c r="A149" t="s">
         <v>153</v>
       </c>
@@ -6154,7 +6145,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:7">
       <c r="A150" t="s">
         <v>154</v>
       </c>
@@ -6174,7 +6165,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:7">
       <c r="A151" t="s">
         <v>155</v>
       </c>
@@ -6194,7 +6185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:7">
       <c r="A152" t="s">
         <v>156</v>
       </c>
@@ -6214,7 +6205,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:7">
       <c r="A153" t="s">
         <v>157</v>
       </c>
@@ -6234,7 +6225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:7">
       <c r="A154" t="s">
         <v>158</v>
       </c>
@@ -6254,7 +6245,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:7">
       <c r="A155" t="s">
         <v>159</v>
       </c>
@@ -6274,7 +6265,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:7">
       <c r="A156" t="s">
         <v>160</v>
       </c>
@@ -6294,7 +6285,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:7">
       <c r="A157" t="s">
         <v>161</v>
       </c>
@@ -6314,7 +6305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:7">
       <c r="A158" t="s">
         <v>162</v>
       </c>
@@ -6334,7 +6325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:7">
       <c r="A159" t="s">
         <v>163</v>
       </c>
@@ -6354,7 +6345,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:7">
       <c r="A160" t="s">
         <v>164</v>
       </c>
@@ -6374,7 +6365,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:7">
       <c r="A161" t="s">
         <v>165</v>
       </c>
@@ -6394,7 +6385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7">
       <c r="A162" t="s">
         <v>166</v>
       </c>
@@ -6414,7 +6405,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:7">
       <c r="A163" t="s">
         <v>167</v>
       </c>
@@ -6434,7 +6425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7">
       <c r="A164" t="s">
         <v>168</v>
       </c>
@@ -6454,7 +6445,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:7">
       <c r="A165" t="s">
         <v>169</v>
       </c>
@@ -6474,7 +6465,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:7">
       <c r="A166" t="s">
         <v>170</v>
       </c>
@@ -6494,7 +6485,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:7">
       <c r="A167" t="s">
         <v>171</v>
       </c>
@@ -6514,7 +6505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:7">
       <c r="A168" t="s">
         <v>172</v>
       </c>
@@ -6534,7 +6525,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:7">
       <c r="A169" t="s">
         <v>173</v>
       </c>
@@ -6554,7 +6545,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:7">
       <c r="A170" t="s">
         <v>174</v>
       </c>
@@ -6574,7 +6565,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:7">
       <c r="A171" t="s">
         <v>175</v>
       </c>
@@ -6594,7 +6585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:7">
       <c r="A172" t="s">
         <v>176</v>
       </c>
@@ -6614,7 +6605,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:7">
       <c r="A173" t="s">
         <v>177</v>
       </c>
@@ -6634,7 +6625,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:7">
       <c r="A174" t="s">
         <v>178</v>
       </c>
@@ -6654,7 +6645,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:7">
       <c r="A175" t="s">
         <v>179</v>
       </c>
@@ -6674,7 +6665,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:7">
       <c r="A176" t="s">
         <v>180</v>
       </c>
@@ -6694,7 +6685,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:7">
       <c r="A177" t="s">
         <v>181</v>
       </c>
@@ -6714,7 +6705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:7">
       <c r="A178" t="s">
         <v>182</v>
       </c>
@@ -6734,7 +6725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:7">
       <c r="A179" t="s">
         <v>183</v>
       </c>
@@ -6754,7 +6745,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:7">
       <c r="A180" t="s">
         <v>184</v>
       </c>
@@ -6774,7 +6765,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:7">
       <c r="A181" t="s">
         <v>185</v>
       </c>
@@ -6794,7 +6785,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:7">
       <c r="A182" t="s">
         <v>186</v>
       </c>
@@ -6814,7 +6805,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:7">
       <c r="A183" t="s">
         <v>187</v>
       </c>
@@ -6834,7 +6825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:7">
       <c r="A184" t="s">
         <v>188</v>
       </c>
@@ -6854,7 +6845,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:7">
       <c r="A185" t="s">
         <v>189</v>
       </c>
@@ -6874,7 +6865,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:7">
       <c r="A186" t="s">
         <v>190</v>
       </c>
@@ -6894,7 +6885,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:7">
       <c r="A187" t="s">
         <v>191</v>
       </c>
@@ -6914,7 +6905,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:7">
       <c r="A188" t="s">
         <v>192</v>
       </c>
@@ -6934,7 +6925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:7">
       <c r="A189" t="s">
         <v>193</v>
       </c>
@@ -6954,7 +6945,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:7">
       <c r="A190" t="s">
         <v>194</v>
       </c>
@@ -6974,7 +6965,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:7">
       <c r="A191" t="s">
         <v>195</v>
       </c>
@@ -6994,7 +6985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:7">
       <c r="A192" t="s">
         <v>196</v>
       </c>
@@ -7014,7 +7005,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:7">
       <c r="A193" t="s">
         <v>197</v>
       </c>
@@ -7034,7 +7025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:7">
       <c r="A194" t="s">
         <v>198</v>
       </c>
@@ -7054,7 +7045,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:7">
       <c r="A195" t="s">
         <v>199</v>
       </c>
@@ -7074,7 +7065,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:7">
       <c r="A196" t="s">
         <v>200</v>
       </c>
@@ -7094,7 +7085,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:7">
       <c r="A197" t="s">
         <v>201</v>
       </c>
@@ -7114,7 +7105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:7">
       <c r="A198" t="s">
         <v>202</v>
       </c>
@@ -7134,7 +7125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:7">
       <c r="A199" t="s">
         <v>203</v>
       </c>
@@ -7154,7 +7145,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:7">
       <c r="A200" t="s">
         <v>204</v>
       </c>
@@ -7174,7 +7165,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:7">
       <c r="A201" t="s">
         <v>205</v>
       </c>
@@ -7194,7 +7185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:7">
       <c r="A202" t="s">
         <v>206</v>
       </c>
@@ -7214,7 +7205,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:7">
       <c r="A203" t="s">
         <v>207</v>
       </c>
@@ -7234,7 +7225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:7">
       <c r="A204" t="s">
         <v>208</v>
       </c>
@@ -7254,7 +7245,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:7">
       <c r="A205" t="s">
         <v>209</v>
       </c>
@@ -7274,7 +7265,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:7">
       <c r="A206" t="s">
         <v>210</v>
       </c>
@@ -7294,7 +7285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:7">
       <c r="A207" t="s">
         <v>211</v>
       </c>
@@ -7314,7 +7305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:7">
       <c r="A208" t="s">
         <v>212</v>
       </c>
@@ -7334,7 +7325,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:7">
       <c r="A209" t="s">
         <v>213</v>
       </c>
@@ -7354,7 +7345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:7">
       <c r="A210" t="s">
         <v>214</v>
       </c>
@@ -7374,7 +7365,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:7">
       <c r="A211" t="s">
         <v>215</v>
       </c>
@@ -7394,7 +7385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:7">
       <c r="A212" t="s">
         <v>216</v>
       </c>
@@ -7414,7 +7405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:7">
       <c r="A213" t="s">
         <v>217</v>
       </c>
@@ -7434,7 +7425,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:7">
       <c r="A214" t="s">
         <v>218</v>
       </c>
@@ -7454,7 +7445,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:7">
       <c r="A215" t="s">
         <v>219</v>
       </c>
@@ -7474,7 +7465,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:7">
       <c r="A216" t="s">
         <v>220</v>
       </c>
@@ -7494,7 +7485,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:7">
       <c r="A217" t="s">
         <v>221</v>
       </c>
@@ -7514,7 +7505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:7">
       <c r="A218" t="s">
         <v>222</v>
       </c>
@@ -7534,7 +7525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:7">
       <c r="A219" t="s">
         <v>223</v>
       </c>
@@ -7554,7 +7545,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:7">
       <c r="A220" t="s">
         <v>224</v>
       </c>
@@ -7574,7 +7565,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:7">
       <c r="A221" t="s">
         <v>225</v>
       </c>
@@ -7594,7 +7585,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:7">
       <c r="A222" t="s">
         <v>226</v>
       </c>
@@ -7614,7 +7605,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:7">
       <c r="A223" t="s">
         <v>227</v>
       </c>
@@ -7634,7 +7625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:7">
       <c r="A224" t="s">
         <v>228</v>
       </c>
@@ -7654,7 +7645,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:7">
       <c r="A225" t="s">
         <v>229</v>
       </c>
@@ -7674,7 +7665,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:7">
       <c r="A226" t="s">
         <v>230</v>
       </c>
@@ -7694,7 +7685,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:7">
       <c r="A227" t="s">
         <v>231</v>
       </c>
@@ -7714,7 +7705,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:7">
       <c r="A228" t="s">
         <v>232</v>
       </c>
@@ -7734,7 +7725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:7">
       <c r="A229" t="s">
         <v>233</v>
       </c>
@@ -7754,7 +7745,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:7">
       <c r="A230" t="s">
         <v>234</v>
       </c>
@@ -7774,7 +7765,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:7">
       <c r="A231" t="s">
         <v>235</v>
       </c>
@@ -7794,7 +7785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:7">
       <c r="A232" t="s">
         <v>236</v>
       </c>
@@ -7814,7 +7805,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:7">
       <c r="A233" t="s">
         <v>237</v>
       </c>
@@ -7834,7 +7825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:7">
       <c r="A234" t="s">
         <v>238</v>
       </c>
@@ -7854,7 +7845,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:7">
       <c r="A235" t="s">
         <v>239</v>
       </c>
@@ -7874,7 +7865,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:7">
       <c r="A236" t="s">
         <v>240</v>
       </c>
@@ -7894,7 +7885,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:7">
       <c r="A237" t="s">
         <v>241</v>
       </c>
@@ -7914,7 +7905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:7">
       <c r="A238" t="s">
         <v>242</v>
       </c>
@@ -7934,7 +7925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:7">
       <c r="A239" t="s">
         <v>243</v>
       </c>
@@ -7954,7 +7945,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:7">
       <c r="A240" t="s">
         <v>244</v>
       </c>
@@ -7974,7 +7965,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:7">
       <c r="A241" t="s">
         <v>245</v>
       </c>
@@ -7994,7 +7985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:7">
       <c r="A242" t="s">
         <v>246</v>
       </c>
@@ -8014,7 +8005,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:7">
       <c r="A243" t="s">
         <v>247</v>
       </c>
@@ -8034,7 +8025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:7">
       <c r="A244" t="s">
         <v>248</v>
       </c>
@@ -8054,7 +8045,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:7">
       <c r="A245" t="s">
         <v>249</v>
       </c>
@@ -8074,7 +8065,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:7">
       <c r="A246" t="s">
         <v>250</v>
       </c>
@@ -8094,7 +8085,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:7">
       <c r="A247" t="s">
         <v>251</v>
       </c>
@@ -8114,7 +8105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:7">
       <c r="A248" t="s">
         <v>252</v>
       </c>
@@ -8134,7 +8125,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:7">
       <c r="A249" t="s">
         <v>253</v>
       </c>
@@ -8154,7 +8145,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:7">
       <c r="A250" t="s">
         <v>254</v>
       </c>
@@ -8174,7 +8165,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:7">
       <c r="A251" t="s">
         <v>255</v>
       </c>
@@ -8194,7 +8185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:7">
       <c r="A252" t="s">
         <v>256</v>
       </c>
@@ -8214,7 +8205,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:7">
       <c r="A253" t="s">
         <v>257</v>
       </c>
@@ -8234,7 +8225,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:7">
       <c r="A254" t="s">
         <v>258</v>
       </c>
@@ -8254,7 +8245,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:7">
       <c r="A255" t="s">
         <v>259</v>
       </c>
@@ -8274,7 +8265,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:7">
       <c r="A256" t="s">
         <v>260</v>
       </c>
@@ -8294,7 +8285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:7">
       <c r="A257" t="s">
         <v>261</v>
       </c>
@@ -8314,7 +8305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:7">
       <c r="A258" t="s">
         <v>262</v>
       </c>
@@ -8334,7 +8325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:7">
       <c r="A259" t="s">
         <v>263</v>
       </c>
@@ -8354,7 +8345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:7">
       <c r="A260" t="s">
         <v>264</v>
       </c>
@@ -8374,7 +8365,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:7">
       <c r="A261" t="s">
         <v>265</v>
       </c>
@@ -8394,7 +8385,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:7">
       <c r="A262" t="s">
         <v>266</v>
       </c>
@@ -8414,7 +8405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:7">
       <c r="A263" t="s">
         <v>267</v>
       </c>
@@ -8434,7 +8425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:7">
       <c r="A264" t="s">
         <v>268</v>
       </c>
@@ -8454,7 +8445,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:7">
       <c r="A265" t="s">
         <v>269</v>
       </c>
@@ -8474,7 +8465,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:7">
       <c r="A266" t="s">
         <v>270</v>
       </c>
@@ -8494,7 +8485,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:7">
       <c r="A267" t="s">
         <v>271</v>
       </c>
@@ -8514,7 +8505,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:7">
       <c r="A268" t="s">
         <v>272</v>
       </c>
@@ -8534,7 +8525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:7">
       <c r="A269" t="s">
         <v>273</v>
       </c>
@@ -8554,7 +8545,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:7">
       <c r="A270" t="s">
         <v>274</v>
       </c>
@@ -8574,7 +8565,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:7">
       <c r="A271" t="s">
         <v>275</v>
       </c>
@@ -8594,7 +8585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:7">
       <c r="A272" t="s">
         <v>276</v>
       </c>
@@ -8614,7 +8605,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:7">
       <c r="A273" t="s">
         <v>277</v>
       </c>
@@ -8634,7 +8625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:7">
       <c r="A274" t="s">
         <v>278</v>
       </c>
@@ -8654,7 +8645,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:7">
       <c r="A275" t="s">
         <v>279</v>
       </c>
@@ -8674,7 +8665,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:7">
       <c r="A276" t="s">
         <v>280</v>
       </c>
@@ -8694,7 +8685,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:7">
       <c r="A277" t="s">
         <v>281</v>
       </c>
@@ -8714,7 +8705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:7">
       <c r="A278" t="s">
         <v>282</v>
       </c>
@@ -8734,7 +8725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:7">
       <c r="A279" t="s">
         <v>283</v>
       </c>
@@ -8754,7 +8745,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:7">
       <c r="A280" t="s">
         <v>284</v>
       </c>
@@ -8774,7 +8765,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:7">
       <c r="A281" t="s">
         <v>285</v>
       </c>
@@ -8794,7 +8785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:7">
       <c r="A282" t="s">
         <v>286</v>
       </c>
@@ -8814,7 +8805,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:7">
       <c r="A283" t="s">
         <v>287</v>
       </c>
@@ -8834,7 +8825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:7">
       <c r="A284" t="s">
         <v>288</v>
       </c>
@@ -8854,7 +8845,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:7">
       <c r="A285" t="s">
         <v>289</v>
       </c>
@@ -8874,7 +8865,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:7">
       <c r="A286" t="s">
         <v>290</v>
       </c>
@@ -8894,7 +8885,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:7">
       <c r="A287" t="s">
         <v>291</v>
       </c>
@@ -8914,7 +8905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:7">
       <c r="A288" t="s">
         <v>292</v>
       </c>
@@ -8934,7 +8925,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:7">
       <c r="A289" t="s">
         <v>293</v>
       </c>
@@ -8954,7 +8945,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:7">
       <c r="A290" t="s">
         <v>294</v>
       </c>
@@ -8974,7 +8965,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:7">
       <c r="A291" t="s">
         <v>295</v>
       </c>
@@ -8994,7 +8985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:7">
       <c r="A292" t="s">
         <v>296</v>
       </c>
@@ -9014,7 +9005,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:7">
       <c r="A293" t="s">
         <v>297</v>
       </c>
@@ -9034,7 +9025,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:7">
       <c r="A294" t="s">
         <v>298</v>
       </c>
@@ -9054,7 +9045,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:7">
       <c r="A295" t="s">
         <v>299</v>
       </c>
@@ -9074,7 +9065,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:7">
       <c r="A296" t="s">
         <v>300</v>
       </c>
@@ -9094,7 +9085,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:7">
       <c r="A297" t="s">
         <v>301</v>
       </c>
@@ -9114,7 +9105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:7">
       <c r="A298" t="s">
         <v>302</v>
       </c>
@@ -9134,7 +9125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:7">
       <c r="A299" t="s">
         <v>303</v>
       </c>
@@ -9154,7 +9145,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:7">
       <c r="A300" t="s">
         <v>304</v>
       </c>
@@ -9174,7 +9165,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:7">
       <c r="A301" t="s">
         <v>305</v>
       </c>
@@ -9194,7 +9185,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:7">
       <c r="A302" t="s">
         <v>306</v>
       </c>
@@ -9214,7 +9205,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:7">
       <c r="A303" t="s">
         <v>307</v>
       </c>
@@ -9234,7 +9225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:7">
       <c r="A304" t="s">
         <v>308</v>
       </c>
@@ -9254,7 +9245,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:7">
       <c r="A305" t="s">
         <v>309</v>
       </c>
@@ -9274,7 +9265,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:7">
       <c r="A306" t="s">
         <v>310</v>
       </c>
@@ -9294,7 +9285,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:7">
       <c r="A307" t="s">
         <v>311</v>
       </c>
@@ -9314,7 +9305,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:7">
       <c r="A308" t="s">
         <v>312</v>
       </c>
@@ -9334,7 +9325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:7">
       <c r="A309" t="s">
         <v>313</v>
       </c>
@@ -9354,7 +9345,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:7">
       <c r="A310" t="s">
         <v>314</v>
       </c>
@@ -9374,7 +9365,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:7">
       <c r="A311" t="s">
         <v>315</v>
       </c>
@@ -9394,7 +9385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:7">
       <c r="A312" t="s">
         <v>316</v>
       </c>
@@ -9414,7 +9405,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:7">
       <c r="A313" t="s">
         <v>317</v>
       </c>
@@ -9434,7 +9425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:7">
       <c r="A314" t="s">
         <v>318</v>
       </c>
@@ -9454,7 +9445,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:7">
       <c r="A315" t="s">
         <v>319</v>
       </c>
@@ -9474,7 +9465,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:7">
       <c r="A316" t="s">
         <v>320</v>
       </c>
@@ -9494,7 +9485,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:7">
       <c r="A317" t="s">
         <v>321</v>
       </c>
@@ -9514,7 +9505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="318" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:7">
       <c r="A318" t="s">
         <v>322</v>
       </c>
@@ -9534,7 +9525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:7">
       <c r="A319" t="s">
         <v>323</v>
       </c>
@@ -9554,7 +9545,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:7">
       <c r="A320" t="s">
         <v>324</v>
       </c>
@@ -9574,7 +9565,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="321" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:7">
       <c r="A321" t="s">
         <v>325</v>
       </c>
@@ -9594,7 +9585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:7">
       <c r="A322" t="s">
         <v>326</v>
       </c>
@@ -9614,7 +9605,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="323" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:7">
       <c r="A323" t="s">
         <v>327</v>
       </c>
@@ -9634,7 +9625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="324" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:7">
       <c r="A324" t="s">
         <v>328</v>
       </c>
@@ -9654,7 +9645,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="325" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:7">
       <c r="A325" t="s">
         <v>329</v>
       </c>
@@ -9674,7 +9665,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="326" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:7">
       <c r="A326" t="s">
         <v>330</v>
       </c>
@@ -9694,7 +9685,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="327" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:7">
       <c r="A327" t="s">
         <v>331</v>
       </c>
@@ -9714,7 +9705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="328" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:7">
       <c r="A328" t="s">
         <v>332</v>
       </c>
@@ -9734,7 +9725,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="329" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:7">
       <c r="A329" t="s">
         <v>333</v>
       </c>
@@ -9754,7 +9745,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="330" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:7">
       <c r="A330" t="s">
         <v>334</v>
       </c>
@@ -9774,7 +9765,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="331" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:7">
       <c r="A331" t="s">
         <v>335</v>
       </c>
@@ -9794,7 +9785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="332" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:7">
       <c r="A332" t="s">
         <v>336</v>
       </c>
@@ -9814,7 +9805,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="333" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:7">
       <c r="A333" t="s">
         <v>337</v>
       </c>
@@ -9834,7 +9825,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="334" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:7">
       <c r="A334" t="s">
         <v>338</v>
       </c>
@@ -9854,7 +9845,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="335" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:7">
       <c r="A335" t="s">
         <v>339</v>
       </c>
@@ -9874,7 +9865,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="336" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:7">
       <c r="A336" t="s">
         <v>340</v>
       </c>
@@ -9894,7 +9885,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="337" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:7">
       <c r="A337" t="s">
         <v>341</v>
       </c>
@@ -9914,7 +9905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="338" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:7">
       <c r="A338" t="s">
         <v>342</v>
       </c>
@@ -9934,7 +9925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="339" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:7">
       <c r="A339" t="s">
         <v>343</v>
       </c>
@@ -9954,7 +9945,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="340" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:7">
       <c r="A340" t="s">
         <v>344</v>
       </c>
@@ -9974,7 +9965,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="341" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:7">
       <c r="A341" t="s">
         <v>345</v>
       </c>
@@ -9994,7 +9985,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="342" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:7">
       <c r="A342" t="s">
         <v>346</v>
       </c>
@@ -10014,7 +10005,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="343" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:7">
       <c r="A343" t="s">
         <v>347</v>
       </c>
@@ -10034,7 +10025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="344" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:7">
       <c r="A344" t="s">
         <v>348</v>
       </c>
@@ -10054,7 +10045,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="345" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:7">
       <c r="A345" t="s">
         <v>349</v>
       </c>
@@ -10074,7 +10065,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="346" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:7">
       <c r="A346" t="s">
         <v>350</v>
       </c>
@@ -10094,7 +10085,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="347" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:7">
       <c r="A347" t="s">
         <v>351</v>
       </c>
@@ -10114,7 +10105,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="348" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:7">
       <c r="A348" t="s">
         <v>352</v>
       </c>
@@ -10134,7 +10125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="349" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:7">
       <c r="A349" t="s">
         <v>353</v>
       </c>
@@ -10154,7 +10145,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="350" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:7">
       <c r="A350" t="s">
         <v>354</v>
       </c>
@@ -10174,7 +10165,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="351" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:7">
       <c r="A351" t="s">
         <v>355</v>
       </c>
@@ -10194,7 +10185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="352" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:7">
       <c r="A352" t="s">
         <v>356</v>
       </c>
@@ -10214,7 +10205,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="353" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:7">
       <c r="A353" t="s">
         <v>357</v>
       </c>
@@ -10234,7 +10225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="354" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:7">
       <c r="A354" t="s">
         <v>358</v>
       </c>
@@ -10254,7 +10245,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="355" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:7">
       <c r="A355" t="s">
         <v>359</v>
       </c>
@@ -10274,7 +10265,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="356" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:7">
       <c r="A356" t="s">
         <v>360</v>
       </c>
@@ -10294,7 +10285,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="357" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:7">
       <c r="A357" t="s">
         <v>361</v>
       </c>
@@ -10314,7 +10305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="358" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:7">
       <c r="A358" t="s">
         <v>362</v>
       </c>
@@ -10334,7 +10325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="359" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:7">
       <c r="A359" t="s">
         <v>363</v>
       </c>
@@ -10354,7 +10345,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="360" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:7">
       <c r="A360" t="s">
         <v>364</v>
       </c>
@@ -10374,7 +10365,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="361" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:7">
       <c r="A361" t="s">
         <v>365</v>
       </c>
@@ -10394,7 +10385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="362" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:7">
       <c r="A362" t="s">
         <v>366</v>
       </c>
@@ -10414,7 +10405,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="363" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:7">
       <c r="A363" t="s">
         <v>367</v>
       </c>
@@ -10434,7 +10425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="364" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:7">
       <c r="A364" t="s">
         <v>368</v>
       </c>
@@ -10454,7 +10445,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="365" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:7">
       <c r="A365" t="s">
         <v>369</v>
       </c>
@@ -10474,7 +10465,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="366" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:7">
       <c r="A366" t="s">
         <v>370</v>
       </c>
@@ -10494,7 +10485,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="367" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:7">
       <c r="A367" t="s">
         <v>371</v>
       </c>
@@ -10514,7 +10505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="368" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:7">
       <c r="A368" t="s">
         <v>372</v>
       </c>
@@ -10534,7 +10525,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="369" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:7">
       <c r="A369" t="s">
         <v>373</v>
       </c>
@@ -10554,7 +10545,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="370" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:7">
       <c r="A370" t="s">
         <v>374</v>
       </c>
@@ -10574,7 +10565,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="371" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:7">
       <c r="A371" t="s">
         <v>375</v>
       </c>
@@ -10594,7 +10585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="372" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:7">
       <c r="A372" t="s">
         <v>376</v>
       </c>
@@ -10614,7 +10605,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="373" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:7">
       <c r="A373" t="s">
         <v>377</v>
       </c>
@@ -10634,7 +10625,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="374" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:7">
       <c r="A374" t="s">
         <v>378</v>
       </c>
@@ -10654,7 +10645,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="375" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:7">
       <c r="A375" t="s">
         <v>379</v>
       </c>
@@ -10674,7 +10665,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="376" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:7">
       <c r="A376" t="s">
         <v>380</v>
       </c>
@@ -10694,7 +10685,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="377" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:7">
       <c r="A377" t="s">
         <v>381</v>
       </c>
@@ -10714,7 +10705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="378" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:7">
       <c r="A378" t="s">
         <v>382</v>
       </c>
@@ -10734,7 +10725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="379" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:7">
       <c r="A379" t="s">
         <v>383</v>
       </c>
@@ -10754,7 +10745,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="380" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:7">
       <c r="A380" t="s">
         <v>384</v>
       </c>
@@ -10774,7 +10765,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="381" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:7">
       <c r="A381" t="s">
         <v>385</v>
       </c>
@@ -10794,7 +10785,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="382" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:7">
       <c r="A382" t="s">
         <v>386</v>
       </c>
@@ -10814,7 +10805,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="383" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:7">
       <c r="A383" t="s">
         <v>387</v>
       </c>
@@ -10834,7 +10825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="384" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:7">
       <c r="A384" t="s">
         <v>388</v>
       </c>
@@ -10854,7 +10845,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="385" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:7">
       <c r="A385" t="s">
         <v>389</v>
       </c>
@@ -10874,7 +10865,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="386" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:7">
       <c r="A386" t="s">
         <v>390</v>
       </c>
@@ -10894,7 +10885,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="387" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:7">
       <c r="A387" t="s">
         <v>391</v>
       </c>
@@ -10914,7 +10905,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="388" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:7">
       <c r="A388" t="s">
         <v>392</v>
       </c>
@@ -10934,7 +10925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="389" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:7">
       <c r="A389" t="s">
         <v>393</v>
       </c>
@@ -10954,7 +10945,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="390" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:7">
       <c r="A390" t="s">
         <v>394</v>
       </c>
@@ -10974,7 +10965,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="391" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:7">
       <c r="A391" t="s">
         <v>395</v>
       </c>
@@ -10994,7 +10985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="392" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:7">
       <c r="A392" t="s">
         <v>396</v>
       </c>
@@ -11014,7 +11005,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="393" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:7">
       <c r="A393" t="s">
         <v>397</v>
       </c>
@@ -11034,7 +11025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="394" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:7">
       <c r="A394" t="s">
         <v>398</v>
       </c>
@@ -11054,7 +11045,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="395" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:7">
       <c r="A395" t="s">
         <v>399</v>
       </c>
@@ -11074,7 +11065,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="396" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:7">
       <c r="A396" t="s">
         <v>400</v>
       </c>
@@ -11094,7 +11085,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="397" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:7">
       <c r="A397" t="s">
         <v>401</v>
       </c>
@@ -11114,7 +11105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="398" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:7">
       <c r="A398" t="s">
         <v>402</v>
       </c>
@@ -11134,7 +11125,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="399" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:7">
       <c r="A399" t="s">
         <v>403</v>
       </c>
@@ -11154,7 +11145,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="400" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:7">
       <c r="A400" t="s">
         <v>404</v>
       </c>
@@ -11174,7 +11165,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="401" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:7">
       <c r="A401" t="s">
         <v>405</v>
       </c>
@@ -11194,7 +11185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="402" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:7">
       <c r="A402" t="s">
         <v>406</v>
       </c>
@@ -11214,7 +11205,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="403" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:7">
       <c r="A403" t="s">
         <v>407</v>
       </c>
@@ -11234,7 +11225,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="404" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:7">
       <c r="A404" t="s">
         <v>408</v>
       </c>
@@ -11254,7 +11245,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="405" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:7">
       <c r="A405" t="s">
         <v>409</v>
       </c>
@@ -11274,7 +11265,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="406" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:7">
       <c r="A406" t="s">
         <v>410</v>
       </c>
@@ -11294,7 +11285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="407" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:7">
       <c r="A407" t="s">
         <v>411</v>
       </c>
@@ -11314,7 +11305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="408" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:7">
       <c r="A408" t="s">
         <v>412</v>
       </c>
@@ -11334,7 +11325,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="409" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:7">
       <c r="A409" t="s">
         <v>413</v>
       </c>
@@ -11354,7 +11345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="410" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:7">
       <c r="A410" t="s">
         <v>414</v>
       </c>
@@ -11374,7 +11365,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="411" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:7">
       <c r="A411" t="s">
         <v>415</v>
       </c>
@@ -11394,7 +11385,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="412" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:7">
       <c r="A412" t="s">
         <v>416</v>
       </c>
@@ -11414,7 +11405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="413" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:7">
       <c r="A413" t="s">
         <v>417</v>
       </c>
@@ -11434,7 +11425,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="414" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:7">
       <c r="A414" t="s">
         <v>418</v>
       </c>
@@ -11454,7 +11445,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="415" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:7">
       <c r="A415" t="s">
         <v>419</v>
       </c>
@@ -11474,7 +11465,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="416" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:7">
       <c r="A416" t="s">
         <v>420</v>
       </c>
@@ -11494,7 +11485,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="417" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:7">
       <c r="A417" t="s">
         <v>421</v>
       </c>
@@ -11514,7 +11505,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="418" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:7">
       <c r="A418" t="s">
         <v>422</v>
       </c>
@@ -11534,7 +11525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="419" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:7">
       <c r="A419" t="s">
         <v>423</v>
       </c>
@@ -11554,7 +11545,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="420" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:7">
       <c r="A420" t="s">
         <v>424</v>
       </c>
@@ -11574,7 +11565,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="421" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:7">
       <c r="A421" t="s">
         <v>425</v>
       </c>
@@ -11594,7 +11585,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="422" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:7">
       <c r="A422" t="s">
         <v>426</v>
       </c>
@@ -11614,7 +11605,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="423" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:7">
       <c r="A423" t="s">
         <v>427</v>
       </c>
@@ -11634,7 +11625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="424" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:7">
       <c r="A424" t="s">
         <v>428</v>
       </c>
@@ -11654,7 +11645,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="425" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:7">
       <c r="A425" t="s">
         <v>429</v>
       </c>
@@ -11674,7 +11665,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="426" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:7">
       <c r="A426" t="s">
         <v>430</v>
       </c>
@@ -11694,7 +11685,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="427" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:7">
       <c r="A427" t="s">
         <v>431</v>
       </c>
@@ -11714,7 +11705,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="428" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:7">
       <c r="A428" t="s">
         <v>432</v>
       </c>
@@ -11734,7 +11725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="429" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:7">
       <c r="A429" t="s">
         <v>433</v>
       </c>
@@ -11754,7 +11745,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="430" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:7">
       <c r="A430" t="s">
         <v>434</v>
       </c>
@@ -11774,7 +11765,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="431" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:7">
       <c r="A431" t="s">
         <v>435</v>
       </c>
@@ -11794,7 +11785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="432" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:7">
       <c r="A432" t="s">
         <v>436</v>
       </c>
@@ -11814,7 +11805,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="433" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:7">
       <c r="A433" t="s">
         <v>437</v>
       </c>
@@ -11834,7 +11825,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="434" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:7">
       <c r="A434" t="s">
         <v>438</v>
       </c>
@@ -11854,7 +11845,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="435" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:7">
       <c r="A435" t="s">
         <v>439</v>
       </c>
@@ -11874,7 +11865,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="436" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:7">
       <c r="A436" t="s">
         <v>440</v>
       </c>
@@ -11894,7 +11885,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="437" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:7">
       <c r="A437" t="s">
         <v>441</v>
       </c>
@@ -11914,7 +11905,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="438" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:7">
       <c r="A438" t="s">
         <v>442</v>
       </c>
@@ -11934,7 +11925,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="439" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:7">
       <c r="A439" t="s">
         <v>443</v>
       </c>
@@ -11954,7 +11945,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="440" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:7">
       <c r="A440" t="s">
         <v>444</v>
       </c>
@@ -11974,7 +11965,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="441" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:7">
       <c r="A441" t="s">
         <v>445</v>
       </c>
@@ -11994,7 +11985,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="442" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:7">
       <c r="A442" t="s">
         <v>446</v>
       </c>
@@ -12014,7 +12005,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="443" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:7">
       <c r="A443" t="s">
         <v>447</v>
       </c>
@@ -12034,7 +12025,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="444" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:7">
       <c r="A444" t="s">
         <v>448</v>
       </c>
@@ -12054,7 +12045,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="445" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:7">
       <c r="A445" t="s">
         <v>449</v>
       </c>
@@ -12074,7 +12065,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="446" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:7">
       <c r="A446" t="s">
         <v>450</v>
       </c>
@@ -12094,7 +12085,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="447" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:7">
       <c r="A447" t="s">
         <v>451</v>
       </c>
@@ -12114,7 +12105,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="448" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:7">
       <c r="A448" t="s">
         <v>452</v>
       </c>
@@ -12134,7 +12125,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="449" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:7">
       <c r="A449" t="s">
         <v>453</v>
       </c>
@@ -12154,7 +12145,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="450" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:7">
       <c r="A450" t="s">
         <v>454</v>
       </c>
@@ -12174,7 +12165,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="451" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:7">
       <c r="A451" t="s">
         <v>455</v>
       </c>
@@ -12194,7 +12185,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="452" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:7">
       <c r="A452" t="s">
         <v>456</v>
       </c>
@@ -12214,7 +12205,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="453" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:7">
       <c r="A453" t="s">
         <v>457</v>
       </c>
@@ -12234,7 +12225,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="454" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:7">
       <c r="A454" t="s">
         <v>458</v>
       </c>
@@ -12254,7 +12245,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="455" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:7">
       <c r="A455" t="s">
         <v>459</v>
       </c>
@@ -12274,7 +12265,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="456" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:7">
       <c r="A456" t="s">
         <v>460</v>
       </c>
@@ -12294,7 +12285,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="457" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:7">
       <c r="A457" t="s">
         <v>461</v>
       </c>
@@ -12314,7 +12305,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="458" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:7">
       <c r="A458" t="s">
         <v>462</v>
       </c>
@@ -12334,7 +12325,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="459" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:7">
       <c r="A459" t="s">
         <v>463</v>
       </c>
@@ -12354,7 +12345,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="460" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:7">
       <c r="A460" t="s">
         <v>464</v>
       </c>
@@ -12374,7 +12365,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="461" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:7">
       <c r="A461" t="s">
         <v>465</v>
       </c>
@@ -12394,7 +12385,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="462" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:7">
       <c r="A462" t="s">
         <v>466</v>
       </c>
@@ -12414,7 +12405,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="463" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:7">
       <c r="A463" t="s">
         <v>467</v>
       </c>
@@ -12434,7 +12425,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="464" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:7">
       <c r="A464" t="s">
         <v>468</v>
       </c>
@@ -12454,7 +12445,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="465" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:7">
       <c r="A465" t="s">
         <v>469</v>
       </c>
@@ -12474,7 +12465,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="466" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:7">
       <c r="A466" t="s">
         <v>470</v>
       </c>
@@ -12494,7 +12485,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="467" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:7">
       <c r="A467" t="s">
         <v>471</v>
       </c>
@@ -12514,7 +12505,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="468" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:7">
       <c r="A468" t="s">
         <v>472</v>
       </c>
@@ -12534,7 +12525,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="469" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:7">
       <c r="A469" t="s">
         <v>473</v>
       </c>
@@ -12554,7 +12545,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="470" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:7">
       <c r="A470" t="s">
         <v>474</v>
       </c>
@@ -12574,7 +12565,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="471" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:7">
       <c r="A471" t="s">
         <v>475</v>
       </c>
@@ -12594,7 +12585,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="472" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:7">
       <c r="A472" t="s">
         <v>476</v>
       </c>
@@ -12614,7 +12605,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="473" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:7">
       <c r="A473" t="s">
         <v>477</v>
       </c>
@@ -12634,7 +12625,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="474" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:7">
       <c r="A474" t="s">
         <v>478</v>
       </c>
@@ -12654,7 +12645,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="475" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:7">
       <c r="A475" t="s">
         <v>479</v>
       </c>
@@ -12674,7 +12665,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="476" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:7">
       <c r="A476" t="s">
         <v>480</v>
       </c>
@@ -12694,7 +12685,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="477" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:7">
       <c r="A477" t="s">
         <v>481</v>
       </c>
@@ -12714,7 +12705,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="478" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:7">
       <c r="A478" t="s">
         <v>482</v>
       </c>
@@ -12734,7 +12725,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="479" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:7">
       <c r="A479" t="s">
         <v>483</v>
       </c>
@@ -12754,7 +12745,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="480" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:7">
       <c r="A480" t="s">
         <v>895</v>
       </c>
@@ -12774,7 +12765,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="481" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:7">
       <c r="A481" t="s">
         <v>896</v>
       </c>
@@ -12794,7 +12785,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="482" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:7">
       <c r="A482" t="s">
         <v>897</v>
       </c>
@@ -12814,7 +12805,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="483" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:7">
       <c r="A483" t="s">
         <v>898</v>
       </c>

</xml_diff>